<commit_message>
🔒 [FULL] Daily chip data 2026-05-29 01:20
</commit_message>
<xml_diff>
--- a/data/reports/chip_radar_2026-05-28.xlsx
+++ b/data/reports/chip_radar_2026-05-28.xlsx
@@ -9115,118 +9115,324 @@
           <t>9217</t>
         </is>
       </c>
-      <c r="D244" s="7" t="inlineStr">
-        <is>
-          <t>⚪ 此分點今日未搶漲停</t>
-        </is>
-      </c>
-      <c r="E244" s="3" t="n"/>
-      <c r="F244" s="3" t="n"/>
-      <c r="G244" s="3" t="n"/>
-      <c r="H244" s="3" t="n"/>
-      <c r="I244" s="3" t="n"/>
-      <c r="J244" s="4" t="n"/>
-      <c r="K244" s="4" t="n"/>
-      <c r="L244" s="5" t="n"/>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>頎邦(6147)</t>
+        </is>
+      </c>
+      <c r="E244" s="3" t="n">
+        <v>10395</v>
+      </c>
+      <c r="F244" s="3" t="n">
+        <v>393</v>
+      </c>
+      <c r="G244" s="3" t="n">
+        <v>302438</v>
+      </c>
+      <c r="H244" s="3" t="n">
+        <v>11254</v>
+      </c>
+      <c r="I244" s="3" t="n">
+        <v>291184</v>
+      </c>
+      <c r="J244" s="4" t="n">
+        <v>290.95</v>
+      </c>
+      <c r="K244" s="4" t="n">
+        <v>286.37</v>
+      </c>
+      <c r="L244" s="6">
+        <f>F244*(K244-J244)</f>
+        <v/>
+      </c>
     </row>
     <row r="245" ht="16.5" customHeight="1">
-      <c r="D245" s="2" t="n"/>
-      <c r="E245" s="3" t="n"/>
-      <c r="F245" s="3" t="n"/>
-      <c r="G245" s="3" t="n"/>
-      <c r="H245" s="3" t="n"/>
-      <c r="I245" s="3" t="n"/>
-      <c r="J245" s="4" t="n"/>
-      <c r="K245" s="4" t="n"/>
-      <c r="L245" s="5" t="n"/>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>聯電(2303)</t>
+        </is>
+      </c>
+      <c r="E245" s="3" t="n">
+        <v>1159</v>
+      </c>
+      <c r="F245" s="3" t="n">
+        <v>1022</v>
+      </c>
+      <c r="G245" s="3" t="n">
+        <v>16858</v>
+      </c>
+      <c r="H245" s="3" t="n">
+        <v>14734</v>
+      </c>
+      <c r="I245" s="3" t="n">
+        <v>2124</v>
+      </c>
+      <c r="J245" s="4" t="n">
+        <v>145.45</v>
+      </c>
+      <c r="K245" s="4" t="n">
+        <v>144.17</v>
+      </c>
+      <c r="L245" s="6">
+        <f>F245*(K245-J245)</f>
+        <v/>
+      </c>
     </row>
     <row r="246" ht="16.5" customHeight="1">
-      <c r="D246" s="2" t="n"/>
-      <c r="E246" s="3" t="n"/>
-      <c r="F246" s="3" t="n"/>
-      <c r="G246" s="3" t="n"/>
-      <c r="H246" s="3" t="n"/>
-      <c r="I246" s="3" t="n"/>
-      <c r="J246" s="4" t="n"/>
-      <c r="K246" s="4" t="n"/>
-      <c r="L246" s="5" t="n"/>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>群創(3481)</t>
+        </is>
+      </c>
+      <c r="E246" s="3" t="n">
+        <v>1295</v>
+      </c>
+      <c r="F246" s="3" t="n">
+        <v>532</v>
+      </c>
+      <c r="G246" s="3" t="n">
+        <v>6336</v>
+      </c>
+      <c r="H246" s="3" t="n">
+        <v>2641</v>
+      </c>
+      <c r="I246" s="3" t="n">
+        <v>3695</v>
+      </c>
+      <c r="J246" s="4" t="n">
+        <v>48.93</v>
+      </c>
+      <c r="K246" s="4" t="n">
+        <v>49.65</v>
+      </c>
+      <c r="L246" s="5">
+        <f>F246*(K246-J246)</f>
+        <v/>
+      </c>
     </row>
     <row r="247" ht="16.5" customHeight="1">
-      <c r="D247" s="2" t="n"/>
-      <c r="E247" s="3" t="n"/>
-      <c r="F247" s="3" t="n"/>
-      <c r="G247" s="3" t="n"/>
-      <c r="H247" s="3" t="n"/>
-      <c r="I247" s="3" t="n"/>
-      <c r="J247" s="4" t="n"/>
-      <c r="K247" s="4" t="n"/>
-      <c r="L247" s="5" t="n"/>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>華邦電(2344)</t>
+        </is>
+      </c>
+      <c r="E247" s="3" t="n">
+        <v>356</v>
+      </c>
+      <c r="F247" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="G247" s="3" t="n">
+        <v>5402</v>
+      </c>
+      <c r="H247" s="3" t="n">
+        <v>1431</v>
+      </c>
+      <c r="I247" s="3" t="n">
+        <v>3971</v>
+      </c>
+      <c r="J247" s="4" t="n">
+        <v>151.74</v>
+      </c>
+      <c r="K247" s="4" t="n">
+        <v>150.62</v>
+      </c>
+      <c r="L247" s="6">
+        <f>F247*(K247-J247)</f>
+        <v/>
+      </c>
     </row>
     <row r="248" ht="16.5" customHeight="1">
-      <c r="D248" s="2" t="n"/>
-      <c r="E248" s="3" t="n"/>
-      <c r="F248" s="3" t="n"/>
-      <c r="G248" s="3" t="n"/>
-      <c r="H248" s="3" t="n"/>
-      <c r="I248" s="3" t="n"/>
-      <c r="J248" s="4" t="n"/>
-      <c r="K248" s="4" t="n"/>
-      <c r="L248" s="5" t="n"/>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>華通(2313)</t>
+        </is>
+      </c>
+      <c r="E248" s="3" t="n">
+        <v>119</v>
+      </c>
+      <c r="F248" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G248" s="3" t="n">
+        <v>3234</v>
+      </c>
+      <c r="H248" s="3" t="n">
+        <v>1154</v>
+      </c>
+      <c r="I248" s="3" t="n">
+        <v>2080</v>
+      </c>
+      <c r="J248" s="4" t="n">
+        <v>271.75</v>
+      </c>
+      <c r="K248" s="4" t="n">
+        <v>268.4</v>
+      </c>
+      <c r="L248" s="6">
+        <f>F248*(K248-J248)</f>
+        <v/>
+      </c>
     </row>
     <row r="249" ht="16.5" customHeight="1">
-      <c r="D249" s="2" t="n"/>
-      <c r="E249" s="3" t="n"/>
-      <c r="F249" s="3" t="n"/>
-      <c r="G249" s="3" t="n"/>
-      <c r="H249" s="3" t="n"/>
-      <c r="I249" s="3" t="n"/>
-      <c r="J249" s="4" t="n"/>
-      <c r="K249" s="4" t="n"/>
-      <c r="L249" s="5" t="n"/>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>台達電(2308)</t>
+        </is>
+      </c>
+      <c r="E249" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F249" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G249" s="3" t="n">
+        <v>2952</v>
+      </c>
+      <c r="H249" s="3" t="n">
+        <v>271</v>
+      </c>
+      <c r="I249" s="3" t="n">
+        <v>2681</v>
+      </c>
+      <c r="J249" s="4" t="n">
+        <v>2460.42</v>
+      </c>
+      <c r="K249" s="4" t="n">
+        <v>2713</v>
+      </c>
+      <c r="L249" s="5">
+        <f>F249*(K249-J249)</f>
+        <v/>
+      </c>
     </row>
     <row r="250" ht="16.5" customHeight="1">
-      <c r="D250" s="2" t="n"/>
-      <c r="E250" s="3" t="n"/>
-      <c r="F250" s="3" t="n"/>
-      <c r="G250" s="3" t="n"/>
-      <c r="H250" s="3" t="n"/>
-      <c r="I250" s="3" t="n"/>
-      <c r="J250" s="4" t="n"/>
-      <c r="K250" s="4" t="n"/>
-      <c r="L250" s="5" t="n"/>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>台光電(2383)</t>
+        </is>
+      </c>
+      <c r="E250" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F250" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G250" s="3" t="n">
+        <v>2234</v>
+      </c>
+      <c r="H250" s="3" t="n">
+        <v>1529</v>
+      </c>
+      <c r="I250" s="3" t="n">
+        <v>705</v>
+      </c>
+      <c r="J250" s="4" t="n">
+        <v>5585</v>
+      </c>
+      <c r="K250" s="4" t="n">
+        <v>5097</v>
+      </c>
+      <c r="L250" s="6">
+        <f>F250*(K250-J250)</f>
+        <v/>
+      </c>
     </row>
     <row r="251" ht="16.5" customHeight="1">
-      <c r="D251" s="2" t="n"/>
-      <c r="E251" s="3" t="n"/>
-      <c r="F251" s="3" t="n"/>
-      <c r="G251" s="3" t="n"/>
-      <c r="H251" s="3" t="n"/>
-      <c r="I251" s="3" t="n"/>
-      <c r="J251" s="4" t="n"/>
-      <c r="K251" s="4" t="n"/>
-      <c r="L251" s="5" t="n"/>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>順德(2351)</t>
+        </is>
+      </c>
+      <c r="E251" s="3" t="n">
+        <v>84</v>
+      </c>
+      <c r="F251" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G251" s="3" t="n">
+        <v>1905</v>
+      </c>
+      <c r="H251" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="I251" s="3" t="n">
+        <v>1859</v>
+      </c>
+      <c r="J251" s="4" t="n">
+        <v>226.79</v>
+      </c>
+      <c r="K251" s="4" t="n">
+        <v>228.5</v>
+      </c>
+      <c r="L251" s="5">
+        <f>F251*(K251-J251)</f>
+        <v/>
+      </c>
     </row>
     <row r="252" ht="16.5" customHeight="1">
-      <c r="D252" s="2" t="n"/>
-      <c r="E252" s="3" t="n"/>
-      <c r="F252" s="3" t="n"/>
-      <c r="G252" s="3" t="n"/>
-      <c r="H252" s="3" t="n"/>
-      <c r="I252" s="3" t="n"/>
-      <c r="J252" s="4" t="n"/>
-      <c r="K252" s="4" t="n"/>
-      <c r="L252" s="5" t="n"/>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>南電(8046)</t>
+        </is>
+      </c>
+      <c r="E252" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="F252" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G252" s="3" t="n">
+        <v>1760</v>
+      </c>
+      <c r="H252" s="3" t="n">
+        <v>454</v>
+      </c>
+      <c r="I252" s="3" t="n">
+        <v>1306</v>
+      </c>
+      <c r="J252" s="4" t="n">
+        <v>838.29</v>
+      </c>
+      <c r="K252" s="4" t="n">
+        <v>907.4</v>
+      </c>
+      <c r="L252" s="5">
+        <f>F252*(K252-J252)</f>
+        <v/>
+      </c>
     </row>
     <row r="253" ht="16.5" customHeight="1">
-      <c r="D253" s="2" t="n"/>
-      <c r="E253" s="3" t="n"/>
-      <c r="F253" s="3" t="n"/>
-      <c r="G253" s="3" t="n"/>
-      <c r="H253" s="3" t="n"/>
-      <c r="I253" s="3" t="n"/>
-      <c r="J253" s="4" t="n"/>
-      <c r="K253" s="4" t="n"/>
-      <c r="L253" s="5" t="n"/>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>華城(1519)</t>
+        </is>
+      </c>
+      <c r="E253" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="F253" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G253" s="3" t="n">
+        <v>1530</v>
+      </c>
+      <c r="H253" s="3" t="n">
+        <v>544</v>
+      </c>
+      <c r="I253" s="3" t="n">
+        <v>986</v>
+      </c>
+      <c r="J253" s="4" t="n">
+        <v>849.72</v>
+      </c>
+      <c r="K253" s="4" t="n">
+        <v>907.5</v>
+      </c>
+      <c r="L253" s="5">
+        <f>F253*(K253-J253)</f>
+        <v/>
+      </c>
     </row>
     <row r="254" ht="16.5" customHeight="1">
       <c r="B254" s="1" t="inlineStr">
@@ -9298,29 +9504,29 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>南茂(8150)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E255" s="3" t="n">
-        <v>12568</v>
+        <v>5493</v>
       </c>
       <c r="F255" s="3" t="n">
-        <v>2235</v>
+        <v>5093</v>
       </c>
       <c r="G255" s="3" t="n">
-        <v>129450</v>
+        <v>181539</v>
       </c>
       <c r="H255" s="3" t="n">
-        <v>23013</v>
+        <v>165197</v>
       </c>
       <c r="I255" s="3" t="n">
-        <v>106437</v>
+        <v>16342</v>
       </c>
       <c r="J255" s="4" t="n">
-        <v>103</v>
+        <v>330.49</v>
       </c>
       <c r="K255" s="4" t="n">
-        <v>102.97</v>
+        <v>324.36</v>
       </c>
       <c r="L255" s="6">
         <f>F255*(K255-J255)</f>
@@ -9330,31 +9536,31 @@
     <row r="256" ht="16.5" customHeight="1">
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>凱美(2375)</t>
+          <t>南茂(8150)</t>
         </is>
       </c>
       <c r="E256" s="3" t="n">
-        <v>600</v>
+        <v>12568</v>
       </c>
       <c r="F256" s="3" t="n">
-        <v>333</v>
+        <v>2235</v>
       </c>
       <c r="G256" s="3" t="n">
-        <v>9689</v>
+        <v>129450</v>
       </c>
       <c r="H256" s="3" t="n">
-        <v>5378</v>
+        <v>23013</v>
       </c>
       <c r="I256" s="3" t="n">
-        <v>4311</v>
+        <v>106437</v>
       </c>
       <c r="J256" s="4" t="n">
-        <v>161.49</v>
+        <v>103</v>
       </c>
       <c r="K256" s="4" t="n">
-        <v>161.5</v>
-      </c>
-      <c r="L256" s="5">
+        <v>102.97</v>
+      </c>
+      <c r="L256" s="6">
         <f>F256*(K256-J256)</f>
         <v/>
       </c>
@@ -9362,29 +9568,29 @@
     <row r="257" ht="16.5" customHeight="1">
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>吉茂(1587)</t>
+          <t>聯發科(2454)</t>
         </is>
       </c>
       <c r="E257" s="3" t="n">
-        <v>668</v>
+        <v>202</v>
       </c>
       <c r="F257" s="3" t="n">
-        <v>4</v>
+        <v>74</v>
       </c>
       <c r="G257" s="3" t="n">
-        <v>2144</v>
+        <v>88901</v>
       </c>
       <c r="H257" s="3" t="n">
-        <v>13</v>
+        <v>32426</v>
       </c>
       <c r="I257" s="3" t="n">
-        <v>2131</v>
+        <v>56475</v>
       </c>
       <c r="J257" s="4" t="n">
-        <v>32.1</v>
+        <v>4401.06</v>
       </c>
       <c r="K257" s="4" t="n">
-        <v>32</v>
+        <v>4381.85</v>
       </c>
       <c r="L257" s="6">
         <f>F257*(K257-J257)</f>
@@ -9392,85 +9598,228 @@
       </c>
     </row>
     <row r="258" ht="16.5" customHeight="1">
-      <c r="D258" s="7" t="inlineStr">
-        <is>
-          <t>⚪ 今日漲停僅 3 檔</t>
-        </is>
-      </c>
-      <c r="E258" s="3" t="n"/>
-      <c r="F258" s="3" t="n"/>
-      <c r="G258" s="3" t="n"/>
-      <c r="H258" s="3" t="n"/>
-      <c r="I258" s="3" t="n"/>
-      <c r="J258" s="4" t="n"/>
-      <c r="K258" s="4" t="n"/>
-      <c r="L258" s="5" t="n"/>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>華南金(2880)</t>
+        </is>
+      </c>
+      <c r="E258" s="3" t="n">
+        <v>17933</v>
+      </c>
+      <c r="F258" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G258" s="3" t="n">
+        <v>53826</v>
+      </c>
+      <c r="H258" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I258" s="3" t="n">
+        <v>53826</v>
+      </c>
+      <c r="J258" s="4" t="n">
+        <v>30.02</v>
+      </c>
+      <c r="K258" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L258" s="5">
+        <f>F258*(K258-J258)</f>
+        <v/>
+      </c>
     </row>
     <row r="259" ht="16.5" customHeight="1">
-      <c r="D259" s="2" t="n"/>
-      <c r="E259" s="3" t="n"/>
-      <c r="F259" s="3" t="n"/>
-      <c r="G259" s="3" t="n"/>
-      <c r="H259" s="3" t="n"/>
-      <c r="I259" s="3" t="n"/>
-      <c r="J259" s="4" t="n"/>
-      <c r="K259" s="4" t="n"/>
-      <c r="L259" s="5" t="n"/>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>長榮航(2618)</t>
+        </is>
+      </c>
+      <c r="E259" s="3" t="n">
+        <v>14527</v>
+      </c>
+      <c r="F259" s="3" t="n">
+        <v>405</v>
+      </c>
+      <c r="G259" s="3" t="n">
+        <v>52025</v>
+      </c>
+      <c r="H259" s="3" t="n">
+        <v>1442</v>
+      </c>
+      <c r="I259" s="3" t="n">
+        <v>50583</v>
+      </c>
+      <c r="J259" s="4" t="n">
+        <v>35.81</v>
+      </c>
+      <c r="K259" s="4" t="n">
+        <v>35.61</v>
+      </c>
+      <c r="L259" s="6">
+        <f>F259*(K259-J259)</f>
+        <v/>
+      </c>
     </row>
     <row r="260" ht="16.5" customHeight="1">
-      <c r="D260" s="2" t="n"/>
-      <c r="E260" s="3" t="n"/>
-      <c r="F260" s="3" t="n"/>
-      <c r="G260" s="3" t="n"/>
-      <c r="H260" s="3" t="n"/>
-      <c r="I260" s="3" t="n"/>
-      <c r="J260" s="4" t="n"/>
-      <c r="K260" s="4" t="n"/>
-      <c r="L260" s="5" t="n"/>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>華碩(2357)</t>
+        </is>
+      </c>
+      <c r="E260" s="3" t="n">
+        <v>687</v>
+      </c>
+      <c r="F260" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G260" s="3" t="n">
+        <v>48175</v>
+      </c>
+      <c r="H260" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I260" s="3" t="n">
+        <v>48175</v>
+      </c>
+      <c r="J260" s="4" t="n">
+        <v>701.23</v>
+      </c>
+      <c r="K260" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L260" s="5">
+        <f>F260*(K260-J260)</f>
+        <v/>
+      </c>
     </row>
     <row r="261" ht="16.5" customHeight="1">
-      <c r="D261" s="2" t="n"/>
-      <c r="E261" s="3" t="n"/>
-      <c r="F261" s="3" t="n"/>
-      <c r="G261" s="3" t="n"/>
-      <c r="H261" s="3" t="n"/>
-      <c r="I261" s="3" t="n"/>
-      <c r="J261" s="4" t="n"/>
-      <c r="K261" s="4" t="n"/>
-      <c r="L261" s="5" t="n"/>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>環球晶(6488)</t>
+        </is>
+      </c>
+      <c r="E261" s="3" t="n">
+        <v>474</v>
+      </c>
+      <c r="F261" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G261" s="3" t="n">
+        <v>46806</v>
+      </c>
+      <c r="H261" s="3" t="n">
+        <v>3302</v>
+      </c>
+      <c r="I261" s="3" t="n">
+        <v>43504</v>
+      </c>
+      <c r="J261" s="4" t="n">
+        <v>987.47</v>
+      </c>
+      <c r="K261" s="4" t="n">
+        <v>943.4299999999999</v>
+      </c>
+      <c r="L261" s="6">
+        <f>F261*(K261-J261)</f>
+        <v/>
+      </c>
     </row>
     <row r="262" ht="16.5" customHeight="1">
-      <c r="D262" s="2" t="n"/>
-      <c r="E262" s="3" t="n"/>
-      <c r="F262" s="3" t="n"/>
-      <c r="G262" s="3" t="n"/>
-      <c r="H262" s="3" t="n"/>
-      <c r="I262" s="3" t="n"/>
-      <c r="J262" s="4" t="n"/>
-      <c r="K262" s="4" t="n"/>
-      <c r="L262" s="5" t="n"/>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>技嘉(2376)</t>
+        </is>
+      </c>
+      <c r="E262" s="3" t="n">
+        <v>1378</v>
+      </c>
+      <c r="F262" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G262" s="3" t="n">
+        <v>46737</v>
+      </c>
+      <c r="H262" s="3" t="n">
+        <v>1274</v>
+      </c>
+      <c r="I262" s="3" t="n">
+        <v>45463</v>
+      </c>
+      <c r="J262" s="4" t="n">
+        <v>339.17</v>
+      </c>
+      <c r="K262" s="4" t="n">
+        <v>335.13</v>
+      </c>
+      <c r="L262" s="6">
+        <f>F262*(K262-J262)</f>
+        <v/>
+      </c>
     </row>
     <row r="263" ht="16.5" customHeight="1">
-      <c r="D263" s="2" t="n"/>
-      <c r="E263" s="3" t="n"/>
-      <c r="F263" s="3" t="n"/>
-      <c r="G263" s="3" t="n"/>
-      <c r="H263" s="3" t="n"/>
-      <c r="I263" s="3" t="n"/>
-      <c r="J263" s="4" t="n"/>
-      <c r="K263" s="4" t="n"/>
-      <c r="L263" s="5" t="n"/>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>台新新光金(2887)</t>
+        </is>
+      </c>
+      <c r="E263" s="3" t="n">
+        <v>17083</v>
+      </c>
+      <c r="F263" s="3" t="n">
+        <v>16064</v>
+      </c>
+      <c r="G263" s="3" t="n">
+        <v>39291</v>
+      </c>
+      <c r="H263" s="3" t="n">
+        <v>36947</v>
+      </c>
+      <c r="I263" s="3" t="n">
+        <v>2344</v>
+      </c>
+      <c r="J263" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="K263" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="L263" s="5">
+        <f>F263*(K263-J263)</f>
+        <v/>
+      </c>
     </row>
     <row r="264" ht="16.5" customHeight="1">
-      <c r="D264" s="2" t="n"/>
-      <c r="E264" s="3" t="n"/>
-      <c r="F264" s="3" t="n"/>
-      <c r="G264" s="3" t="n"/>
-      <c r="H264" s="3" t="n"/>
-      <c r="I264" s="3" t="n"/>
-      <c r="J264" s="4" t="n"/>
-      <c r="K264" s="4" t="n"/>
-      <c r="L264" s="5" t="n"/>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>統一超(2912)</t>
+        </is>
+      </c>
+      <c r="E264" s="3" t="n">
+        <v>1548</v>
+      </c>
+      <c r="F264" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G264" s="3" t="n">
+        <v>32404</v>
+      </c>
+      <c r="H264" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I264" s="3" t="n">
+        <v>32404</v>
+      </c>
+      <c r="J264" s="4" t="n">
+        <v>209.33</v>
+      </c>
+      <c r="K264" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L264" s="5">
+        <f>F264*(K264-J264)</f>
+        <v/>
+      </c>
     </row>
     <row r="265" ht="16.5" customHeight="1">
       <c r="B265" s="1" t="inlineStr">
@@ -9542,29 +9891,29 @@
       </c>
       <c r="D266" s="2" t="inlineStr">
         <is>
-          <t>南茂(8150)</t>
+          <t>力成(6239)</t>
         </is>
       </c>
       <c r="E266" s="3" t="n">
-        <v>11856</v>
+        <v>10828</v>
       </c>
       <c r="F266" s="3" t="n">
-        <v>10673</v>
+        <v>9771</v>
       </c>
       <c r="G266" s="3" t="n">
-        <v>122110</v>
+        <v>402564</v>
       </c>
       <c r="H266" s="3" t="n">
-        <v>109577</v>
+        <v>360454</v>
       </c>
       <c r="I266" s="3" t="n">
-        <v>12533</v>
+        <v>42110</v>
       </c>
       <c r="J266" s="4" t="n">
-        <v>102.99</v>
+        <v>371.78</v>
       </c>
       <c r="K266" s="4" t="n">
-        <v>102.67</v>
+        <v>368.9</v>
       </c>
       <c r="L266" s="6">
         <f>F266*(K266-J266)</f>
@@ -9574,31 +9923,31 @@
     <row r="267" ht="16.5" customHeight="1">
       <c r="D267" s="2" t="inlineStr">
         <is>
-          <t>萬潤(6187)</t>
+          <t>力積電(6770)</t>
         </is>
       </c>
       <c r="E267" s="3" t="n">
-        <v>939</v>
+        <v>42810</v>
       </c>
       <c r="F267" s="3" t="n">
-        <v>64</v>
+        <v>24411</v>
       </c>
       <c r="G267" s="3" t="n">
-        <v>116434</v>
+        <v>345658</v>
       </c>
       <c r="H267" s="3" t="n">
-        <v>7972</v>
+        <v>196211</v>
       </c>
       <c r="I267" s="3" t="n">
-        <v>108462</v>
+        <v>149447</v>
       </c>
       <c r="J267" s="4" t="n">
-        <v>1239.98</v>
+        <v>80.73999999999999</v>
       </c>
       <c r="K267" s="4" t="n">
-        <v>1245.56</v>
-      </c>
-      <c r="L267" s="5">
+        <v>80.38</v>
+      </c>
+      <c r="L267" s="6">
         <f>F267*(K267-J267)</f>
         <v/>
       </c>
@@ -9606,31 +9955,31 @@
     <row r="268" ht="16.5" customHeight="1">
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>立隆電(2472)</t>
+          <t>廣達(2382)</t>
         </is>
       </c>
       <c r="E268" s="3" t="n">
-        <v>1189</v>
+        <v>6457</v>
       </c>
       <c r="F268" s="3" t="n">
-        <v>444</v>
+        <v>189</v>
       </c>
       <c r="G268" s="3" t="n">
-        <v>44104</v>
+        <v>202881</v>
       </c>
       <c r="H268" s="3" t="n">
-        <v>16488</v>
+        <v>5890</v>
       </c>
       <c r="I268" s="3" t="n">
-        <v>27616</v>
+        <v>196991</v>
       </c>
       <c r="J268" s="4" t="n">
-        <v>370.94</v>
+        <v>314.2</v>
       </c>
       <c r="K268" s="4" t="n">
-        <v>371.36</v>
-      </c>
-      <c r="L268" s="5">
+        <v>311.65</v>
+      </c>
+      <c r="L268" s="6">
         <f>F268*(K268-J268)</f>
         <v/>
       </c>
@@ -9638,104 +9987,226 @@
     <row r="269" ht="16.5" customHeight="1">
       <c r="D269" s="2" t="inlineStr">
         <is>
-          <t>凱美(2375)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E269" s="3" t="n">
-        <v>2519</v>
+        <v>5382</v>
       </c>
       <c r="F269" s="3" t="n">
-        <v>630</v>
+        <v>4760</v>
       </c>
       <c r="G269" s="3" t="n">
-        <v>40672</v>
+        <v>174367</v>
       </c>
       <c r="H269" s="3" t="n">
-        <v>10014</v>
+        <v>154236</v>
       </c>
       <c r="I269" s="3" t="n">
-        <v>30658</v>
+        <v>20131</v>
       </c>
       <c r="J269" s="4" t="n">
-        <v>161.46</v>
+        <v>323.98</v>
       </c>
       <c r="K269" s="4" t="n">
-        <v>158.95</v>
-      </c>
-      <c r="L269" s="6">
+        <v>324.03</v>
+      </c>
+      <c r="L269" s="5">
         <f>F269*(K269-J269)</f>
         <v/>
       </c>
     </row>
     <row r="270" ht="16.5" customHeight="1">
-      <c r="D270" s="7" t="inlineStr">
-        <is>
-          <t>⚪ 今日漲停僅 4 檔</t>
-        </is>
-      </c>
-      <c r="E270" s="3" t="n"/>
-      <c r="F270" s="3" t="n"/>
-      <c r="G270" s="3" t="n"/>
-      <c r="H270" s="3" t="n"/>
-      <c r="I270" s="3" t="n"/>
-      <c r="J270" s="4" t="n"/>
-      <c r="K270" s="4" t="n"/>
-      <c r="L270" s="5" t="n"/>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>南茂(8150)</t>
+        </is>
+      </c>
+      <c r="E270" s="3" t="n">
+        <v>11856</v>
+      </c>
+      <c r="F270" s="3" t="n">
+        <v>10673</v>
+      </c>
+      <c r="G270" s="3" t="n">
+        <v>122110</v>
+      </c>
+      <c r="H270" s="3" t="n">
+        <v>109577</v>
+      </c>
+      <c r="I270" s="3" t="n">
+        <v>12533</v>
+      </c>
+      <c r="J270" s="4" t="n">
+        <v>102.99</v>
+      </c>
+      <c r="K270" s="4" t="n">
+        <v>102.67</v>
+      </c>
+      <c r="L270" s="6">
+        <f>F270*(K270-J270)</f>
+        <v/>
+      </c>
     </row>
     <row r="271" ht="16.5" customHeight="1">
-      <c r="D271" s="2" t="n"/>
-      <c r="E271" s="3" t="n"/>
-      <c r="F271" s="3" t="n"/>
-      <c r="G271" s="3" t="n"/>
-      <c r="H271" s="3" t="n"/>
-      <c r="I271" s="3" t="n"/>
-      <c r="J271" s="4" t="n"/>
-      <c r="K271" s="4" t="n"/>
-      <c r="L271" s="5" t="n"/>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>萬潤(6187)</t>
+        </is>
+      </c>
+      <c r="E271" s="3" t="n">
+        <v>939</v>
+      </c>
+      <c r="F271" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="G271" s="3" t="n">
+        <v>116434</v>
+      </c>
+      <c r="H271" s="3" t="n">
+        <v>7972</v>
+      </c>
+      <c r="I271" s="3" t="n">
+        <v>108462</v>
+      </c>
+      <c r="J271" s="4" t="n">
+        <v>1239.98</v>
+      </c>
+      <c r="K271" s="4" t="n">
+        <v>1245.56</v>
+      </c>
+      <c r="L271" s="5">
+        <f>F271*(K271-J271)</f>
+        <v/>
+      </c>
     </row>
     <row r="272" ht="16.5" customHeight="1">
-      <c r="D272" s="2" t="n"/>
-      <c r="E272" s="3" t="n"/>
-      <c r="F272" s="3" t="n"/>
-      <c r="G272" s="3" t="n"/>
-      <c r="H272" s="3" t="n"/>
-      <c r="I272" s="3" t="n"/>
-      <c r="J272" s="4" t="n"/>
-      <c r="K272" s="4" t="n"/>
-      <c r="L272" s="5" t="n"/>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>環球晶(6488)</t>
+        </is>
+      </c>
+      <c r="E272" s="3" t="n">
+        <v>891</v>
+      </c>
+      <c r="F272" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G272" s="3" t="n">
+        <v>85688</v>
+      </c>
+      <c r="H272" s="3" t="n">
+        <v>3492</v>
+      </c>
+      <c r="I272" s="3" t="n">
+        <v>82196</v>
+      </c>
+      <c r="J272" s="4" t="n">
+        <v>961.71</v>
+      </c>
+      <c r="K272" s="4" t="n">
+        <v>969.89</v>
+      </c>
+      <c r="L272" s="5">
+        <f>F272*(K272-J272)</f>
+        <v/>
+      </c>
     </row>
     <row r="273" ht="16.5" customHeight="1">
-      <c r="D273" s="2" t="n"/>
-      <c r="E273" s="3" t="n"/>
-      <c r="F273" s="3" t="n"/>
-      <c r="G273" s="3" t="n"/>
-      <c r="H273" s="3" t="n"/>
-      <c r="I273" s="3" t="n"/>
-      <c r="J273" s="4" t="n"/>
-      <c r="K273" s="4" t="n"/>
-      <c r="L273" s="5" t="n"/>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>致茂(2360)</t>
+        </is>
+      </c>
+      <c r="E273" s="3" t="n">
+        <v>275</v>
+      </c>
+      <c r="F273" s="3" t="n">
+        <v>123</v>
+      </c>
+      <c r="G273" s="3" t="n">
+        <v>70644</v>
+      </c>
+      <c r="H273" s="3" t="n">
+        <v>31485</v>
+      </c>
+      <c r="I273" s="3" t="n">
+        <v>39159</v>
+      </c>
+      <c r="J273" s="4" t="n">
+        <v>2568.88</v>
+      </c>
+      <c r="K273" s="4" t="n">
+        <v>2559.72</v>
+      </c>
+      <c r="L273" s="6">
+        <f>F273*(K273-J273)</f>
+        <v/>
+      </c>
     </row>
     <row r="274" ht="16.5" customHeight="1">
-      <c r="D274" s="2" t="n"/>
-      <c r="E274" s="3" t="n"/>
-      <c r="F274" s="3" t="n"/>
-      <c r="G274" s="3" t="n"/>
-      <c r="H274" s="3" t="n"/>
-      <c r="I274" s="3" t="n"/>
-      <c r="J274" s="4" t="n"/>
-      <c r="K274" s="4" t="n"/>
-      <c r="L274" s="5" t="n"/>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>鴻勁(7769)</t>
+        </is>
+      </c>
+      <c r="E274" s="3" t="n">
+        <v>91</v>
+      </c>
+      <c r="F274" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G274" s="3" t="n">
+        <v>70224</v>
+      </c>
+      <c r="H274" s="3" t="n">
+        <v>19662</v>
+      </c>
+      <c r="I274" s="3" t="n">
+        <v>50562</v>
+      </c>
+      <c r="J274" s="4" t="n">
+        <v>7716.96</v>
+      </c>
+      <c r="K274" s="4" t="n">
+        <v>7562.42</v>
+      </c>
+      <c r="L274" s="6">
+        <f>F274*(K274-J274)</f>
+        <v/>
+      </c>
     </row>
     <row r="275" ht="16.5" customHeight="1">
-      <c r="D275" s="2" t="n"/>
-      <c r="E275" s="3" t="n"/>
-      <c r="F275" s="3" t="n"/>
-      <c r="G275" s="3" t="n"/>
-      <c r="H275" s="3" t="n"/>
-      <c r="I275" s="3" t="n"/>
-      <c r="J275" s="4" t="n"/>
-      <c r="K275" s="4" t="n"/>
-      <c r="L275" s="5" t="n"/>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>群聯(8299)</t>
+        </is>
+      </c>
+      <c r="E275" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="F275" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="G275" s="3" t="n">
+        <v>61318</v>
+      </c>
+      <c r="H275" s="3" t="n">
+        <v>13325</v>
+      </c>
+      <c r="I275" s="3" t="n">
+        <v>47993</v>
+      </c>
+      <c r="J275" s="4" t="n">
+        <v>2452.73</v>
+      </c>
+      <c r="K275" s="4" t="n">
+        <v>2467.54</v>
+      </c>
+      <c r="L275" s="5">
+        <f>F275*(K275-J275)</f>
+        <v/>
+      </c>
     </row>
     <row r="276" ht="16.5" customHeight="1">
       <c r="A276" s="1" t="inlineStr">
@@ -12933,31 +13404,31 @@
       </c>
       <c r="D365" s="2" t="inlineStr">
         <is>
-          <t>東陽(1319)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E365" s="3" t="n">
-        <v>232</v>
+        <v>178</v>
       </c>
       <c r="F365" s="3" t="n">
-        <v>4</v>
+        <v>78</v>
       </c>
       <c r="G365" s="3" t="n">
-        <v>2007</v>
+        <v>5769</v>
       </c>
       <c r="H365" s="3" t="n">
-        <v>33</v>
+        <v>2546</v>
       </c>
       <c r="I365" s="3" t="n">
-        <v>1974</v>
+        <v>3223</v>
       </c>
       <c r="J365" s="4" t="n">
-        <v>86.5</v>
+        <v>324.12</v>
       </c>
       <c r="K365" s="4" t="n">
-        <v>83</v>
-      </c>
-      <c r="L365" s="6">
+        <v>326.38</v>
+      </c>
+      <c r="L365" s="5">
         <f>F365*(K365-J365)</f>
         <v/>
       </c>
@@ -12965,29 +13436,29 @@
     <row r="366" ht="16.5" customHeight="1">
       <c r="D366" s="2" t="inlineStr">
         <is>
-          <t>萬潤(6187)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E366" s="3" t="n">
-        <v>10</v>
+        <v>319</v>
       </c>
       <c r="F366" s="3" t="n">
-        <v>3</v>
+        <v>164</v>
       </c>
       <c r="G366" s="3" t="n">
-        <v>1178</v>
+        <v>4821</v>
       </c>
       <c r="H366" s="3" t="n">
-        <v>337</v>
+        <v>2468</v>
       </c>
       <c r="I366" s="3" t="n">
-        <v>841</v>
+        <v>2353</v>
       </c>
       <c r="J366" s="4" t="n">
-        <v>1178.1</v>
+        <v>151.13</v>
       </c>
       <c r="K366" s="4" t="n">
-        <v>1122.33</v>
+        <v>150.49</v>
       </c>
       <c r="L366" s="6">
         <f>F366*(K366-J366)</f>
@@ -12997,29 +13468,29 @@
     <row r="367" ht="16.5" customHeight="1">
       <c r="D367" s="2" t="inlineStr">
         <is>
-          <t>麗清(3346)</t>
+          <t>環球晶(6488)</t>
         </is>
       </c>
       <c r="E367" s="3" t="n">
-        <v>282</v>
+        <v>47</v>
       </c>
       <c r="F367" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G367" s="3" t="n">
-        <v>550</v>
+        <v>4580</v>
       </c>
       <c r="H367" s="3" t="n">
-        <v>0</v>
+        <v>780</v>
       </c>
       <c r="I367" s="3" t="n">
-        <v>550</v>
+        <v>3800</v>
       </c>
       <c r="J367" s="4" t="n">
-        <v>19.5</v>
+        <v>974.36</v>
       </c>
       <c r="K367" s="4" t="n">
-        <v>0</v>
+        <v>975.62</v>
       </c>
       <c r="L367" s="5">
         <f>F367*(K367-J367)</f>
@@ -13029,31 +13500,31 @@
     <row r="368" ht="16.5" customHeight="1">
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>太欣(5302)</t>
+          <t>群聯(8299)</t>
         </is>
       </c>
       <c r="E368" s="3" t="n">
-        <v>230</v>
+        <v>18</v>
       </c>
       <c r="F368" s="3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G368" s="3" t="n">
-        <v>252</v>
+        <v>4528</v>
       </c>
       <c r="H368" s="3" t="n">
-        <v>0</v>
+        <v>2145</v>
       </c>
       <c r="I368" s="3" t="n">
-        <v>252</v>
+        <v>2383</v>
       </c>
       <c r="J368" s="4" t="n">
-        <v>10.95</v>
+        <v>2515.5</v>
       </c>
       <c r="K368" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L368" s="5">
+        <v>2383.33</v>
+      </c>
+      <c r="L368" s="6">
         <f>F368*(K368-J368)</f>
         <v/>
       </c>
@@ -13061,93 +13532,194 @@
     <row r="369" ht="16.5" customHeight="1">
       <c r="D369" s="2" t="inlineStr">
         <is>
-          <t>昱捷(3232)</t>
+          <t>京元電子(2449)</t>
         </is>
       </c>
       <c r="E369" s="3" t="n">
-        <v>67</v>
+        <v>137</v>
       </c>
       <c r="F369" s="3" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="G369" s="3" t="n">
-        <v>153</v>
+        <v>4480</v>
       </c>
       <c r="H369" s="3" t="n">
-        <v>0</v>
+        <v>1663</v>
       </c>
       <c r="I369" s="3" t="n">
-        <v>153</v>
+        <v>2817</v>
       </c>
       <c r="J369" s="4" t="n">
-        <v>22.9</v>
+        <v>327.01</v>
       </c>
       <c r="K369" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L369" s="5">
+        <v>326.02</v>
+      </c>
+      <c r="L369" s="6">
         <f>F369*(K369-J369)</f>
         <v/>
       </c>
     </row>
     <row r="370" ht="16.5" customHeight="1">
-      <c r="D370" s="7" t="inlineStr">
-        <is>
-          <t>⚪ 今日漲停僅 5 檔</t>
-        </is>
-      </c>
-      <c r="E370" s="3" t="n"/>
-      <c r="F370" s="3" t="n"/>
-      <c r="G370" s="3" t="n"/>
-      <c r="H370" s="3" t="n"/>
-      <c r="I370" s="3" t="n"/>
-      <c r="J370" s="4" t="n"/>
-      <c r="K370" s="4" t="n"/>
-      <c r="L370" s="5" t="n"/>
+      <c r="D370" s="2" t="inlineStr">
+        <is>
+          <t>群創(3481)</t>
+        </is>
+      </c>
+      <c r="E370" s="3" t="n">
+        <v>837</v>
+      </c>
+      <c r="F370" s="3" t="n">
+        <v>314</v>
+      </c>
+      <c r="G370" s="3" t="n">
+        <v>4088</v>
+      </c>
+      <c r="H370" s="3" t="n">
+        <v>1523</v>
+      </c>
+      <c r="I370" s="3" t="n">
+        <v>2565</v>
+      </c>
+      <c r="J370" s="4" t="n">
+        <v>48.85</v>
+      </c>
+      <c r="K370" s="4" t="n">
+        <v>48.51</v>
+      </c>
+      <c r="L370" s="6">
+        <f>F370*(K370-J370)</f>
+        <v/>
+      </c>
     </row>
     <row r="371" ht="16.5" customHeight="1">
-      <c r="D371" s="2" t="n"/>
-      <c r="E371" s="3" t="n"/>
-      <c r="F371" s="3" t="n"/>
-      <c r="G371" s="3" t="n"/>
-      <c r="H371" s="3" t="n"/>
-      <c r="I371" s="3" t="n"/>
-      <c r="J371" s="4" t="n"/>
-      <c r="K371" s="4" t="n"/>
-      <c r="L371" s="5" t="n"/>
+      <c r="D371" s="2" t="inlineStr">
+        <is>
+          <t>信驊(5274)</t>
+        </is>
+      </c>
+      <c r="E371" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F371" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G371" s="3" t="n">
+        <v>3708</v>
+      </c>
+      <c r="H371" s="3" t="n">
+        <v>345</v>
+      </c>
+      <c r="I371" s="3" t="n">
+        <v>3363</v>
+      </c>
+      <c r="J371" s="4" t="n">
+        <v>18537.5</v>
+      </c>
+      <c r="K371" s="4" t="n">
+        <v>3450</v>
+      </c>
+      <c r="L371" s="6">
+        <f>F371*(K371-J371)</f>
+        <v/>
+      </c>
     </row>
     <row r="372" ht="16.5" customHeight="1">
-      <c r="D372" s="2" t="n"/>
-      <c r="E372" s="3" t="n"/>
-      <c r="F372" s="3" t="n"/>
-      <c r="G372" s="3" t="n"/>
-      <c r="H372" s="3" t="n"/>
-      <c r="I372" s="3" t="n"/>
-      <c r="J372" s="4" t="n"/>
-      <c r="K372" s="4" t="n"/>
-      <c r="L372" s="5" t="n"/>
+      <c r="D372" s="2" t="inlineStr">
+        <is>
+          <t>創意(3443)</t>
+        </is>
+      </c>
+      <c r="E372" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F372" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G372" s="3" t="n">
+        <v>3176</v>
+      </c>
+      <c r="H372" s="3" t="n">
+        <v>1204</v>
+      </c>
+      <c r="I372" s="3" t="n">
+        <v>1972</v>
+      </c>
+      <c r="J372" s="4" t="n">
+        <v>4537.43</v>
+      </c>
+      <c r="K372" s="4" t="n">
+        <v>4014.33</v>
+      </c>
+      <c r="L372" s="6">
+        <f>F372*(K372-J372)</f>
+        <v/>
+      </c>
     </row>
     <row r="373" ht="16.5" customHeight="1">
-      <c r="D373" s="2" t="n"/>
-      <c r="E373" s="3" t="n"/>
-      <c r="F373" s="3" t="n"/>
-      <c r="G373" s="3" t="n"/>
-      <c r="H373" s="3" t="n"/>
-      <c r="I373" s="3" t="n"/>
-      <c r="J373" s="4" t="n"/>
-      <c r="K373" s="4" t="n"/>
-      <c r="L373" s="5" t="n"/>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t>聯鈞(3450)</t>
+        </is>
+      </c>
+      <c r="E373" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="F373" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G373" s="3" t="n">
+        <v>2255</v>
+      </c>
+      <c r="H373" s="3" t="n">
+        <v>499</v>
+      </c>
+      <c r="I373" s="3" t="n">
+        <v>1756</v>
+      </c>
+      <c r="J373" s="4" t="n">
+        <v>479.77</v>
+      </c>
+      <c r="K373" s="4" t="n">
+        <v>498.6</v>
+      </c>
+      <c r="L373" s="5">
+        <f>F373*(K373-J373)</f>
+        <v/>
+      </c>
     </row>
     <row r="374" ht="16.5" customHeight="1">
-      <c r="D374" s="2" t="n"/>
-      <c r="E374" s="3" t="n"/>
-      <c r="F374" s="3" t="n"/>
-      <c r="G374" s="3" t="n"/>
-      <c r="H374" s="3" t="n"/>
-      <c r="I374" s="3" t="n"/>
-      <c r="J374" s="4" t="n"/>
-      <c r="K374" s="4" t="n"/>
-      <c r="L374" s="5" t="n"/>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>欣興(3037)</t>
+        </is>
+      </c>
+      <c r="E374" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F374" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="G374" s="3" t="n">
+        <v>2210</v>
+      </c>
+      <c r="H374" s="3" t="n">
+        <v>867</v>
+      </c>
+      <c r="I374" s="3" t="n">
+        <v>1343</v>
+      </c>
+      <c r="J374" s="4" t="n">
+        <v>1004.77</v>
+      </c>
+      <c r="K374" s="4" t="n">
+        <v>1084.12</v>
+      </c>
+      <c r="L374" s="5">
+        <f>F374*(K374-J374)</f>
+        <v/>
+      </c>
     </row>
     <row r="375" ht="16.5" customHeight="1">
       <c r="A375" s="1" t="inlineStr">
@@ -13229,29 +13801,29 @@
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t>南茂(8150)</t>
+          <t>華邦電(2344)</t>
         </is>
       </c>
       <c r="E376" s="3" t="n">
-        <v>1103</v>
+        <v>1770</v>
       </c>
       <c r="F376" s="3" t="n">
-        <v>47</v>
+        <v>1629</v>
       </c>
       <c r="G376" s="3" t="n">
-        <v>11345</v>
+        <v>26824</v>
       </c>
       <c r="H376" s="3" t="n">
-        <v>482</v>
+        <v>24576</v>
       </c>
       <c r="I376" s="3" t="n">
-        <v>10863</v>
+        <v>2248</v>
       </c>
       <c r="J376" s="4" t="n">
-        <v>102.85</v>
+        <v>151.55</v>
       </c>
       <c r="K376" s="4" t="n">
-        <v>102.57</v>
+        <v>150.87</v>
       </c>
       <c r="L376" s="6">
         <f>F376*(K376-J376)</f>
@@ -13261,126 +13833,290 @@
     <row r="377" ht="16.5" customHeight="1">
       <c r="D377" s="2" t="inlineStr">
         <is>
+          <t>力積電(6770)</t>
+        </is>
+      </c>
+      <c r="E377" s="3" t="n">
+        <v>2706</v>
+      </c>
+      <c r="F377" s="3" t="n">
+        <v>532</v>
+      </c>
+      <c r="G377" s="3" t="n">
+        <v>21770</v>
+      </c>
+      <c r="H377" s="3" t="n">
+        <v>4207</v>
+      </c>
+      <c r="I377" s="3" t="n">
+        <v>17563</v>
+      </c>
+      <c r="J377" s="4" t="n">
+        <v>80.45</v>
+      </c>
+      <c r="K377" s="4" t="n">
+        <v>79.08</v>
+      </c>
+      <c r="L377" s="6">
+        <f>F377*(K377-J377)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="378" ht="16.5" customHeight="1">
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t>南茂(8150)</t>
+        </is>
+      </c>
+      <c r="E378" s="3" t="n">
+        <v>1103</v>
+      </c>
+      <c r="F378" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="G378" s="3" t="n">
+        <v>11345</v>
+      </c>
+      <c r="H378" s="3" t="n">
+        <v>482</v>
+      </c>
+      <c r="I378" s="3" t="n">
+        <v>10863</v>
+      </c>
+      <c r="J378" s="4" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="K378" s="4" t="n">
+        <v>102.57</v>
+      </c>
+      <c r="L378" s="6">
+        <f>F378*(K378-J378)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="379" ht="16.5" customHeight="1">
+      <c r="D379" s="2" t="inlineStr">
+        <is>
+          <t>國巨*(2327)</t>
+        </is>
+      </c>
+      <c r="E379" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="F379" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="G379" s="3" t="n">
+        <v>8503</v>
+      </c>
+      <c r="H379" s="3" t="n">
+        <v>2165</v>
+      </c>
+      <c r="I379" s="3" t="n">
+        <v>6338</v>
+      </c>
+      <c r="J379" s="4" t="n">
+        <v>733.03</v>
+      </c>
+      <c r="K379" s="4" t="n">
+        <v>746.41</v>
+      </c>
+      <c r="L379" s="5">
+        <f>F379*(K379-J379)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="380" ht="16.5" customHeight="1">
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t>力成(6239)</t>
+        </is>
+      </c>
+      <c r="E380" s="3" t="n">
+        <v>196</v>
+      </c>
+      <c r="F380" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="G380" s="3" t="n">
+        <v>7181</v>
+      </c>
+      <c r="H380" s="3" t="n">
+        <v>1877</v>
+      </c>
+      <c r="I380" s="3" t="n">
+        <v>5304</v>
+      </c>
+      <c r="J380" s="4" t="n">
+        <v>366.36</v>
+      </c>
+      <c r="K380" s="4" t="n">
+        <v>367.96</v>
+      </c>
+      <c r="L380" s="5">
+        <f>F380*(K380-J380)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="381" ht="16.5" customHeight="1">
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t>頎邦(6147)</t>
+        </is>
+      </c>
+      <c r="E381" s="3" t="n">
+        <v>199</v>
+      </c>
+      <c r="F381" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="G381" s="3" t="n">
+        <v>5554</v>
+      </c>
+      <c r="H381" s="3" t="n">
+        <v>921</v>
+      </c>
+      <c r="I381" s="3" t="n">
+        <v>4633</v>
+      </c>
+      <c r="J381" s="4" t="n">
+        <v>279.1</v>
+      </c>
+      <c r="K381" s="4" t="n">
+        <v>279.12</v>
+      </c>
+      <c r="L381" s="5">
+        <f>F381*(K381-J381)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="382" ht="16.5" customHeight="1">
+      <c r="D382" s="2" t="inlineStr">
+        <is>
           <t>晶技(3042)</t>
         </is>
       </c>
-      <c r="E377" s="3" t="n">
+      <c r="E382" s="3" t="n">
         <v>251</v>
       </c>
-      <c r="F377" s="3" t="n">
+      <c r="F382" s="3" t="n">
         <v>156</v>
       </c>
-      <c r="G377" s="3" t="n">
+      <c r="G382" s="3" t="n">
         <v>5434</v>
       </c>
-      <c r="H377" s="3" t="n">
+      <c r="H382" s="3" t="n">
         <v>3393</v>
       </c>
-      <c r="I377" s="3" t="n">
+      <c r="I382" s="3" t="n">
         <v>2041</v>
       </c>
-      <c r="J377" s="4" t="n">
+      <c r="J382" s="4" t="n">
         <v>216.47</v>
       </c>
-      <c r="K377" s="4" t="n">
+      <c r="K382" s="4" t="n">
         <v>217.47</v>
       </c>
-      <c r="L377" s="5">
-        <f>F377*(K377-J377)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="378" ht="16.5" customHeight="1">
-      <c r="D378" s="7" t="inlineStr">
-        <is>
-          <t>⚪ 今日漲停僅 2 檔</t>
-        </is>
-      </c>
-      <c r="E378" s="3" t="n"/>
-      <c r="F378" s="3" t="n"/>
-      <c r="G378" s="3" t="n"/>
-      <c r="H378" s="3" t="n"/>
-      <c r="I378" s="3" t="n"/>
-      <c r="J378" s="4" t="n"/>
-      <c r="K378" s="4" t="n"/>
-      <c r="L378" s="5" t="n"/>
-    </row>
-    <row r="379" ht="16.5" customHeight="1">
-      <c r="D379" s="2" t="n"/>
-      <c r="E379" s="3" t="n"/>
-      <c r="F379" s="3" t="n"/>
-      <c r="G379" s="3" t="n"/>
-      <c r="H379" s="3" t="n"/>
-      <c r="I379" s="3" t="n"/>
-      <c r="J379" s="4" t="n"/>
-      <c r="K379" s="4" t="n"/>
-      <c r="L379" s="5" t="n"/>
-    </row>
-    <row r="380" ht="16.5" customHeight="1">
-      <c r="D380" s="2" t="n"/>
-      <c r="E380" s="3" t="n"/>
-      <c r="F380" s="3" t="n"/>
-      <c r="G380" s="3" t="n"/>
-      <c r="H380" s="3" t="n"/>
-      <c r="I380" s="3" t="n"/>
-      <c r="J380" s="4" t="n"/>
-      <c r="K380" s="4" t="n"/>
-      <c r="L380" s="5" t="n"/>
-    </row>
-    <row r="381" ht="16.5" customHeight="1">
-      <c r="D381" s="2" t="n"/>
-      <c r="E381" s="3" t="n"/>
-      <c r="F381" s="3" t="n"/>
-      <c r="G381" s="3" t="n"/>
-      <c r="H381" s="3" t="n"/>
-      <c r="I381" s="3" t="n"/>
-      <c r="J381" s="4" t="n"/>
-      <c r="K381" s="4" t="n"/>
-      <c r="L381" s="5" t="n"/>
-    </row>
-    <row r="382" ht="16.5" customHeight="1">
-      <c r="D382" s="2" t="n"/>
-      <c r="E382" s="3" t="n"/>
-      <c r="F382" s="3" t="n"/>
-      <c r="G382" s="3" t="n"/>
-      <c r="H382" s="3" t="n"/>
-      <c r="I382" s="3" t="n"/>
-      <c r="J382" s="4" t="n"/>
-      <c r="K382" s="4" t="n"/>
-      <c r="L382" s="5" t="n"/>
+      <c r="L382" s="5">
+        <f>F382*(K382-J382)</f>
+        <v/>
+      </c>
     </row>
     <row r="383" ht="16.5" customHeight="1">
-      <c r="D383" s="2" t="n"/>
-      <c r="E383" s="3" t="n"/>
-      <c r="F383" s="3" t="n"/>
-      <c r="G383" s="3" t="n"/>
-      <c r="H383" s="3" t="n"/>
-      <c r="I383" s="3" t="n"/>
-      <c r="J383" s="4" t="n"/>
-      <c r="K383" s="4" t="n"/>
-      <c r="L383" s="5" t="n"/>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>台燿(6274)</t>
+        </is>
+      </c>
+      <c r="E383" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F383" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G383" s="3" t="n">
+        <v>5350</v>
+      </c>
+      <c r="H383" s="3" t="n">
+        <v>3394</v>
+      </c>
+      <c r="I383" s="3" t="n">
+        <v>1956</v>
+      </c>
+      <c r="J383" s="4" t="n">
+        <v>1528.46</v>
+      </c>
+      <c r="K383" s="4" t="n">
+        <v>1542.59</v>
+      </c>
+      <c r="L383" s="5">
+        <f>F383*(K383-J383)</f>
+        <v/>
+      </c>
     </row>
     <row r="384" ht="16.5" customHeight="1">
-      <c r="D384" s="2" t="n"/>
-      <c r="E384" s="3" t="n"/>
-      <c r="F384" s="3" t="n"/>
-      <c r="G384" s="3" t="n"/>
-      <c r="H384" s="3" t="n"/>
-      <c r="I384" s="3" t="n"/>
-      <c r="J384" s="4" t="n"/>
-      <c r="K384" s="4" t="n"/>
-      <c r="L384" s="5" t="n"/>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>擎亞(8096)</t>
+        </is>
+      </c>
+      <c r="E384" s="3" t="n">
+        <v>243</v>
+      </c>
+      <c r="F384" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="G384" s="3" t="n">
+        <v>3067</v>
+      </c>
+      <c r="H384" s="3" t="n">
+        <v>165</v>
+      </c>
+      <c r="I384" s="3" t="n">
+        <v>2902</v>
+      </c>
+      <c r="J384" s="4" t="n">
+        <v>126.22</v>
+      </c>
+      <c r="K384" s="4" t="n">
+        <v>127.08</v>
+      </c>
+      <c r="L384" s="5">
+        <f>F384*(K384-J384)</f>
+        <v/>
+      </c>
     </row>
     <row r="385" ht="16.5" customHeight="1">
-      <c r="D385" s="2" t="n"/>
-      <c r="E385" s="3" t="n"/>
-      <c r="F385" s="3" t="n"/>
-      <c r="G385" s="3" t="n"/>
-      <c r="H385" s="3" t="n"/>
-      <c r="I385" s="3" t="n"/>
-      <c r="J385" s="4" t="n"/>
-      <c r="K385" s="4" t="n"/>
-      <c r="L385" s="5" t="n"/>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>智邦(2345)</t>
+        </is>
+      </c>
+      <c r="E385" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="F385" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G385" s="3" t="n">
+        <v>2788</v>
+      </c>
+      <c r="H385" s="3" t="n">
+        <v>752</v>
+      </c>
+      <c r="I385" s="3" t="n">
+        <v>2036</v>
+      </c>
+      <c r="J385" s="4" t="n">
+        <v>2534.09</v>
+      </c>
+      <c r="K385" s="4" t="n">
+        <v>2505.67</v>
+      </c>
+      <c r="L385" s="6">
+        <f>F385*(K385-J385)</f>
+        <v/>
+      </c>
     </row>
     <row r="386" ht="16.5" customHeight="1">
       <c r="B386" s="1" t="inlineStr">
@@ -13452,29 +14188,29 @@
       </c>
       <c r="D387" s="2" t="inlineStr">
         <is>
-          <t>南茂(8150)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E387" s="3" t="n">
-        <v>362</v>
+        <v>3049</v>
       </c>
       <c r="F387" s="3" t="n">
-        <v>241</v>
+        <v>2340</v>
       </c>
       <c r="G387" s="3" t="n">
-        <v>3728</v>
+        <v>15047</v>
       </c>
       <c r="H387" s="3" t="n">
-        <v>2478</v>
+        <v>11492</v>
       </c>
       <c r="I387" s="3" t="n">
-        <v>1250</v>
+        <v>3555</v>
       </c>
       <c r="J387" s="4" t="n">
-        <v>102.98</v>
+        <v>49.35</v>
       </c>
       <c r="K387" s="4" t="n">
-        <v>102.83</v>
+        <v>49.11</v>
       </c>
       <c r="L387" s="6">
         <f>F387*(K387-J387)</f>
@@ -13484,29 +14220,29 @@
     <row r="388" ht="16.5" customHeight="1">
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>興勤(2428)</t>
+          <t>台積電(2330)</t>
         </is>
       </c>
       <c r="E388" s="3" t="n">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="F388" s="3" t="n">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="G388" s="3" t="n">
-        <v>2486</v>
+        <v>10808</v>
       </c>
       <c r="H388" s="3" t="n">
-        <v>1580</v>
+        <v>5752</v>
       </c>
       <c r="I388" s="3" t="n">
-        <v>906</v>
+        <v>5056</v>
       </c>
       <c r="J388" s="4" t="n">
-        <v>292.51</v>
+        <v>2299.49</v>
       </c>
       <c r="K388" s="4" t="n">
-        <v>292.57</v>
+        <v>2300.72</v>
       </c>
       <c r="L388" s="5">
         <f>F388*(K388-J388)</f>
@@ -13516,29 +14252,29 @@
     <row r="389" ht="16.5" customHeight="1">
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>東陽(1319)</t>
+          <t>南亞科(2408)</t>
         </is>
       </c>
       <c r="E389" s="3" t="n">
-        <v>257</v>
+        <v>215</v>
       </c>
       <c r="F389" s="3" t="n">
-        <v>27</v>
+        <v>185</v>
       </c>
       <c r="G389" s="3" t="n">
-        <v>2223</v>
+        <v>6956</v>
       </c>
       <c r="H389" s="3" t="n">
-        <v>234</v>
+        <v>5988</v>
       </c>
       <c r="I389" s="3" t="n">
-        <v>1989</v>
+        <v>968</v>
       </c>
       <c r="J389" s="4" t="n">
-        <v>86.5</v>
+        <v>323.53</v>
       </c>
       <c r="K389" s="4" t="n">
-        <v>86.63</v>
+        <v>323.68</v>
       </c>
       <c r="L389" s="5">
         <f>F389*(K389-J389)</f>
@@ -13548,104 +14284,226 @@
     <row r="390" ht="16.5" customHeight="1">
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>泰藝(8289)</t>
+          <t>聯電(2303)</t>
         </is>
       </c>
       <c r="E390" s="3" t="n">
-        <v>211</v>
+        <v>289</v>
       </c>
       <c r="F390" s="3" t="n">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="G390" s="3" t="n">
-        <v>1596</v>
+        <v>4177</v>
       </c>
       <c r="H390" s="3" t="n">
-        <v>836</v>
+        <v>1829</v>
       </c>
       <c r="I390" s="3" t="n">
+        <v>2348</v>
+      </c>
+      <c r="J390" s="4" t="n">
+        <v>144.54</v>
+      </c>
+      <c r="K390" s="4" t="n">
+        <v>145.17</v>
+      </c>
+      <c r="L390" s="5">
+        <f>F390*(K390-J390)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="391" ht="16.5" customHeight="1">
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>聯發科(2454)</t>
+        </is>
+      </c>
+      <c r="E391" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F391" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G391" s="3" t="n">
+        <v>3825</v>
+      </c>
+      <c r="H391" s="3" t="n">
+        <v>720</v>
+      </c>
+      <c r="I391" s="3" t="n">
+        <v>3105</v>
+      </c>
+      <c r="J391" s="4" t="n">
+        <v>4250</v>
+      </c>
+      <c r="K391" s="4" t="n">
+        <v>3600.5</v>
+      </c>
+      <c r="L391" s="6">
+        <f>F391*(K391-J391)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="392" ht="16.5" customHeight="1">
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>南茂(8150)</t>
+        </is>
+      </c>
+      <c r="E392" s="3" t="n">
+        <v>362</v>
+      </c>
+      <c r="F392" s="3" t="n">
+        <v>241</v>
+      </c>
+      <c r="G392" s="3" t="n">
+        <v>3728</v>
+      </c>
+      <c r="H392" s="3" t="n">
+        <v>2478</v>
+      </c>
+      <c r="I392" s="3" t="n">
+        <v>1250</v>
+      </c>
+      <c r="J392" s="4" t="n">
+        <v>102.98</v>
+      </c>
+      <c r="K392" s="4" t="n">
+        <v>102.83</v>
+      </c>
+      <c r="L392" s="6">
+        <f>F392*(K392-J392)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="393" ht="16.5" customHeight="1">
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>金寶(2312)</t>
+        </is>
+      </c>
+      <c r="E393" s="3" t="n">
+        <v>809</v>
+      </c>
+      <c r="F393" s="3" t="n">
+        <v>598</v>
+      </c>
+      <c r="G393" s="3" t="n">
+        <v>3215</v>
+      </c>
+      <c r="H393" s="3" t="n">
+        <v>2376</v>
+      </c>
+      <c r="I393" s="3" t="n">
+        <v>839</v>
+      </c>
+      <c r="J393" s="4" t="n">
+        <v>39.74</v>
+      </c>
+      <c r="K393" s="4" t="n">
+        <v>39.74</v>
+      </c>
+      <c r="L393" s="5">
+        <f>F393*(K393-J393)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="394" ht="16.5" customHeight="1">
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>矽力*-KY(6415)</t>
+        </is>
+      </c>
+      <c r="E394" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="F394" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G394" s="3" t="n">
+        <v>3147</v>
+      </c>
+      <c r="H394" s="3" t="n">
+        <v>2387</v>
+      </c>
+      <c r="I394" s="3" t="n">
         <v>760</v>
       </c>
-      <c r="J390" s="4" t="n">
-        <v>75.65000000000001</v>
-      </c>
-      <c r="K390" s="4" t="n">
-        <v>75.31999999999999</v>
-      </c>
-      <c r="L390" s="6">
-        <f>F390*(K390-J390)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="391" ht="16.5" customHeight="1">
-      <c r="D391" s="7" t="inlineStr">
-        <is>
-          <t>⚪ 今日漲停僅 4 檔</t>
-        </is>
-      </c>
-      <c r="E391" s="3" t="n"/>
-      <c r="F391" s="3" t="n"/>
-      <c r="G391" s="3" t="n"/>
-      <c r="H391" s="3" t="n"/>
-      <c r="I391" s="3" t="n"/>
-      <c r="J391" s="4" t="n"/>
-      <c r="K391" s="4" t="n"/>
-      <c r="L391" s="5" t="n"/>
-    </row>
-    <row r="392" ht="16.5" customHeight="1">
-      <c r="D392" s="2" t="n"/>
-      <c r="E392" s="3" t="n"/>
-      <c r="F392" s="3" t="n"/>
-      <c r="G392" s="3" t="n"/>
-      <c r="H392" s="3" t="n"/>
-      <c r="I392" s="3" t="n"/>
-      <c r="J392" s="4" t="n"/>
-      <c r="K392" s="4" t="n"/>
-      <c r="L392" s="5" t="n"/>
-    </row>
-    <row r="393" ht="16.5" customHeight="1">
-      <c r="D393" s="2" t="n"/>
-      <c r="E393" s="3" t="n"/>
-      <c r="F393" s="3" t="n"/>
-      <c r="G393" s="3" t="n"/>
-      <c r="H393" s="3" t="n"/>
-      <c r="I393" s="3" t="n"/>
-      <c r="J393" s="4" t="n"/>
-      <c r="K393" s="4" t="n"/>
-      <c r="L393" s="5" t="n"/>
-    </row>
-    <row r="394" ht="16.5" customHeight="1">
-      <c r="D394" s="2" t="n"/>
-      <c r="E394" s="3" t="n"/>
-      <c r="F394" s="3" t="n"/>
-      <c r="G394" s="3" t="n"/>
-      <c r="H394" s="3" t="n"/>
-      <c r="I394" s="3" t="n"/>
-      <c r="J394" s="4" t="n"/>
-      <c r="K394" s="4" t="n"/>
-      <c r="L394" s="5" t="n"/>
+      <c r="J394" s="4" t="n">
+        <v>617.02</v>
+      </c>
+      <c r="K394" s="4" t="n">
+        <v>612.15</v>
+      </c>
+      <c r="L394" s="6">
+        <f>F394*(K394-J394)</f>
+        <v/>
+      </c>
     </row>
     <row r="395" ht="16.5" customHeight="1">
-      <c r="D395" s="2" t="n"/>
-      <c r="E395" s="3" t="n"/>
-      <c r="F395" s="3" t="n"/>
-      <c r="G395" s="3" t="n"/>
-      <c r="H395" s="3" t="n"/>
-      <c r="I395" s="3" t="n"/>
-      <c r="J395" s="4" t="n"/>
-      <c r="K395" s="4" t="n"/>
-      <c r="L395" s="5" t="n"/>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>華通(2313)</t>
+        </is>
+      </c>
+      <c r="E395" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="F395" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G395" s="3" t="n">
+        <v>2543</v>
+      </c>
+      <c r="H395" s="3" t="n">
+        <v>1034</v>
+      </c>
+      <c r="I395" s="3" t="n">
+        <v>1509</v>
+      </c>
+      <c r="J395" s="4" t="n">
+        <v>270.49</v>
+      </c>
+      <c r="K395" s="4" t="n">
+        <v>271.97</v>
+      </c>
+      <c r="L395" s="5">
+        <f>F395*(K395-J395)</f>
+        <v/>
+      </c>
     </row>
     <row r="396" ht="16.5" customHeight="1">
-      <c r="D396" s="2" t="n"/>
-      <c r="E396" s="3" t="n"/>
-      <c r="F396" s="3" t="n"/>
-      <c r="G396" s="3" t="n"/>
-      <c r="H396" s="3" t="n"/>
-      <c r="I396" s="3" t="n"/>
-      <c r="J396" s="4" t="n"/>
-      <c r="K396" s="4" t="n"/>
-      <c r="L396" s="5" t="n"/>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>興勤(2428)</t>
+        </is>
+      </c>
+      <c r="E396" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="F396" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="G396" s="3" t="n">
+        <v>2486</v>
+      </c>
+      <c r="H396" s="3" t="n">
+        <v>1580</v>
+      </c>
+      <c r="I396" s="3" t="n">
+        <v>906</v>
+      </c>
+      <c r="J396" s="4" t="n">
+        <v>292.51</v>
+      </c>
+      <c r="K396" s="4" t="n">
+        <v>292.57</v>
+      </c>
+      <c r="L396" s="5">
+        <f>F396*(K396-J396)</f>
+        <v/>
+      </c>
     </row>
     <row r="397" ht="16.5" customHeight="1">
       <c r="B397" s="1" t="inlineStr">
@@ -13717,29 +14575,29 @@
       </c>
       <c r="D398" s="2" t="inlineStr">
         <is>
-          <t>台半(5425)</t>
+          <t>信驊(5274)</t>
         </is>
       </c>
       <c r="E398" s="3" t="n">
-        <v>88</v>
+        <v>7</v>
       </c>
       <c r="F398" s="3" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="G398" s="3" t="n">
-        <v>955</v>
+        <v>12770</v>
       </c>
       <c r="H398" s="3" t="n">
-        <v>182</v>
+        <v>11192</v>
       </c>
       <c r="I398" s="3" t="n">
-        <v>773</v>
+        <v>1578</v>
       </c>
       <c r="J398" s="4" t="n">
-        <v>108.48</v>
+        <v>18242.86</v>
       </c>
       <c r="K398" s="4" t="n">
-        <v>113.5</v>
+        <v>18653</v>
       </c>
       <c r="L398" s="5">
         <f>F398*(K398-J398)</f>
@@ -13749,29 +14607,29 @@
     <row r="399" ht="16.5" customHeight="1">
       <c r="D399" s="2" t="inlineStr">
         <is>
-          <t>新纖(1409)</t>
+          <t>華通(2313)</t>
         </is>
       </c>
       <c r="E399" s="3" t="n">
-        <v>80</v>
+        <v>309</v>
       </c>
       <c r="F399" s="3" t="n">
-        <v>31</v>
+        <v>195</v>
       </c>
       <c r="G399" s="3" t="n">
-        <v>166</v>
+        <v>8686</v>
       </c>
       <c r="H399" s="3" t="n">
-        <v>64</v>
+        <v>5182</v>
       </c>
       <c r="I399" s="3" t="n">
-        <v>102</v>
+        <v>3504</v>
       </c>
       <c r="J399" s="4" t="n">
-        <v>20.75</v>
+        <v>281.09</v>
       </c>
       <c r="K399" s="4" t="n">
-        <v>20.74</v>
+        <v>265.76</v>
       </c>
       <c r="L399" s="6">
         <f>F399*(K399-J399)</f>
@@ -13781,115 +14639,258 @@
     <row r="400" ht="16.5" customHeight="1">
       <c r="D400" s="2" t="inlineStr">
         <is>
-          <t>國喬(1312)</t>
+          <t>群創(3481)</t>
         </is>
       </c>
       <c r="E400" s="3" t="n">
-        <v>101</v>
+        <v>1529</v>
       </c>
       <c r="F400" s="3" t="n">
-        <v>0</v>
+        <v>441</v>
       </c>
       <c r="G400" s="3" t="n">
-        <v>111</v>
+        <v>7494</v>
       </c>
       <c r="H400" s="3" t="n">
-        <v>0</v>
+        <v>2144</v>
       </c>
       <c r="I400" s="3" t="n">
-        <v>111</v>
+        <v>5350</v>
       </c>
       <c r="J400" s="4" t="n">
-        <v>10.95</v>
+        <v>49.01</v>
       </c>
       <c r="K400" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L400" s="5">
+        <v>48.61</v>
+      </c>
+      <c r="L400" s="6">
         <f>F400*(K400-J400)</f>
         <v/>
       </c>
     </row>
     <row r="401" ht="16.5" customHeight="1">
-      <c r="D401" s="7" t="inlineStr">
-        <is>
-          <t>⚪ 今日漲停僅 3 檔</t>
-        </is>
-      </c>
-      <c r="E401" s="3" t="n"/>
-      <c r="F401" s="3" t="n"/>
-      <c r="G401" s="3" t="n"/>
-      <c r="H401" s="3" t="n"/>
-      <c r="I401" s="3" t="n"/>
-      <c r="J401" s="4" t="n"/>
-      <c r="K401" s="4" t="n"/>
-      <c r="L401" s="5" t="n"/>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>創意(3443)</t>
+        </is>
+      </c>
+      <c r="E401" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="F401" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G401" s="3" t="n">
+        <v>6202</v>
+      </c>
+      <c r="H401" s="3" t="n">
+        <v>527</v>
+      </c>
+      <c r="I401" s="3" t="n">
+        <v>5675</v>
+      </c>
+      <c r="J401" s="4" t="n">
+        <v>4429.79</v>
+      </c>
+      <c r="K401" s="4" t="n">
+        <v>5266</v>
+      </c>
+      <c r="L401" s="5">
+        <f>F401*(K401-J401)</f>
+        <v/>
+      </c>
     </row>
     <row r="402" ht="16.5" customHeight="1">
-      <c r="D402" s="2" t="n"/>
-      <c r="E402" s="3" t="n"/>
-      <c r="F402" s="3" t="n"/>
-      <c r="G402" s="3" t="n"/>
-      <c r="H402" s="3" t="n"/>
-      <c r="I402" s="3" t="n"/>
-      <c r="J402" s="4" t="n"/>
-      <c r="K402" s="4" t="n"/>
-      <c r="L402" s="5" t="n"/>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t>亞翔(6139)</t>
+        </is>
+      </c>
+      <c r="E402" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="F402" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G402" s="3" t="n">
+        <v>5022</v>
+      </c>
+      <c r="H402" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I402" s="3" t="n">
+        <v>5014</v>
+      </c>
+      <c r="J402" s="4" t="n">
+        <v>772.55</v>
+      </c>
+      <c r="K402" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="L402" s="6">
+        <f>F402*(K402-J402)</f>
+        <v/>
+      </c>
     </row>
     <row r="403" ht="16.5" customHeight="1">
-      <c r="D403" s="2" t="n"/>
-      <c r="E403" s="3" t="n"/>
-      <c r="F403" s="3" t="n"/>
-      <c r="G403" s="3" t="n"/>
-      <c r="H403" s="3" t="n"/>
-      <c r="I403" s="3" t="n"/>
-      <c r="J403" s="4" t="n"/>
-      <c r="K403" s="4" t="n"/>
-      <c r="L403" s="5" t="n"/>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t>可成(2474)</t>
+        </is>
+      </c>
+      <c r="E403" s="3" t="n">
+        <v>223</v>
+      </c>
+      <c r="F403" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G403" s="3" t="n">
+        <v>4497</v>
+      </c>
+      <c r="H403" s="3" t="n">
+        <v>687</v>
+      </c>
+      <c r="I403" s="3" t="n">
+        <v>3810</v>
+      </c>
+      <c r="J403" s="4" t="n">
+        <v>201.66</v>
+      </c>
+      <c r="K403" s="4" t="n">
+        <v>196.4</v>
+      </c>
+      <c r="L403" s="6">
+        <f>F403*(K403-J403)</f>
+        <v/>
+      </c>
     </row>
     <row r="404" ht="16.5" customHeight="1">
-      <c r="D404" s="2" t="n"/>
-      <c r="E404" s="3" t="n"/>
-      <c r="F404" s="3" t="n"/>
-      <c r="G404" s="3" t="n"/>
-      <c r="H404" s="3" t="n"/>
-      <c r="I404" s="3" t="n"/>
-      <c r="J404" s="4" t="n"/>
-      <c r="K404" s="4" t="n"/>
-      <c r="L404" s="5" t="n"/>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>台積電(2330)</t>
+        </is>
+      </c>
+      <c r="E404" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F404" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="G404" s="3" t="n">
+        <v>4493</v>
+      </c>
+      <c r="H404" s="3" t="n">
+        <v>3929</v>
+      </c>
+      <c r="I404" s="3" t="n">
+        <v>564</v>
+      </c>
+      <c r="J404" s="4" t="n">
+        <v>2246.35</v>
+      </c>
+      <c r="K404" s="4" t="n">
+        <v>2310.94</v>
+      </c>
+      <c r="L404" s="5">
+        <f>F404*(K404-J404)</f>
+        <v/>
+      </c>
     </row>
     <row r="405" ht="16.5" customHeight="1">
-      <c r="D405" s="2" t="n"/>
-      <c r="E405" s="3" t="n"/>
-      <c r="F405" s="3" t="n"/>
-      <c r="G405" s="3" t="n"/>
-      <c r="H405" s="3" t="n"/>
-      <c r="I405" s="3" t="n"/>
-      <c r="J405" s="4" t="n"/>
-      <c r="K405" s="4" t="n"/>
-      <c r="L405" s="5" t="n"/>
+      <c r="D405" s="2" t="inlineStr">
+        <is>
+          <t>金像電(2368)</t>
+        </is>
+      </c>
+      <c r="E405" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="F405" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G405" s="3" t="n">
+        <v>4030</v>
+      </c>
+      <c r="H405" s="3" t="n">
+        <v>669</v>
+      </c>
+      <c r="I405" s="3" t="n">
+        <v>3361</v>
+      </c>
+      <c r="J405" s="4" t="n">
+        <v>1299.84</v>
+      </c>
+      <c r="K405" s="4" t="n">
+        <v>1337.2</v>
+      </c>
+      <c r="L405" s="5">
+        <f>F405*(K405-J405)</f>
+        <v/>
+      </c>
     </row>
     <row r="406" ht="16.5" customHeight="1">
-      <c r="D406" s="2" t="n"/>
-      <c r="E406" s="3" t="n"/>
-      <c r="F406" s="3" t="n"/>
-      <c r="G406" s="3" t="n"/>
-      <c r="H406" s="3" t="n"/>
-      <c r="I406" s="3" t="n"/>
-      <c r="J406" s="4" t="n"/>
-      <c r="K406" s="4" t="n"/>
-      <c r="L406" s="5" t="n"/>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>華邦電(2344)</t>
+        </is>
+      </c>
+      <c r="E406" s="3" t="n">
+        <v>186</v>
+      </c>
+      <c r="F406" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="G406" s="3" t="n">
+        <v>2808</v>
+      </c>
+      <c r="H406" s="3" t="n">
+        <v>1484</v>
+      </c>
+      <c r="I406" s="3" t="n">
+        <v>1324</v>
+      </c>
+      <c r="J406" s="4" t="n">
+        <v>150.96</v>
+      </c>
+      <c r="K406" s="4" t="n">
+        <v>148.38</v>
+      </c>
+      <c r="L406" s="6">
+        <f>F406*(K406-J406)</f>
+        <v/>
+      </c>
     </row>
     <row r="407" ht="16.5" customHeight="1">
-      <c r="D407" s="2" t="n"/>
-      <c r="E407" s="3" t="n"/>
-      <c r="F407" s="3" t="n"/>
-      <c r="G407" s="3" t="n"/>
-      <c r="H407" s="3" t="n"/>
-      <c r="I407" s="3" t="n"/>
-      <c r="J407" s="4" t="n"/>
-      <c r="K407" s="4" t="n"/>
-      <c r="L407" s="5" t="n"/>
+      <c r="D407" s="2" t="inlineStr">
+        <is>
+          <t>精成科(6191)</t>
+        </is>
+      </c>
+      <c r="E407" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="F407" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G407" s="3" t="n">
+        <v>2605</v>
+      </c>
+      <c r="H407" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="I407" s="3" t="n">
+        <v>2545</v>
+      </c>
+      <c r="J407" s="4" t="n">
+        <v>100.98</v>
+      </c>
+      <c r="K407" s="4" t="n">
+        <v>100.83</v>
+      </c>
+      <c r="L407" s="6">
+        <f>F407*(K407-J407)</f>
+        <v/>
+      </c>
     </row>
     <row r="408" ht="16.5" customHeight="1">
       <c r="A408" s="1" t="inlineStr">

</xml_diff>